<commit_message>
Enhance PDF extraction and KPI parsing for improved accuracy
- Modified `extract_pages` function to accept a `sort` parameter, allowing for text extraction in sorted order when necessary.
- Implemented fallback mechanism in `build_structure` to use sorted text extraction if fewer than 9 principle headers are found, ensuring better recovery of indicators in complex layouts.
- Updated KPI parsing functions to handle variations in text formatting, including adjustments for numeric token recognition and regex patterns for specific phrases.
- Introduced `_sorted_text_for` function to re-extract PDF text with sorted order for cases where default extraction fails to capture necessary data.
</commit_message>
<xml_diff>
--- a/data/output/brsr_deliverables.xlsx
+++ b/data/output/brsr_deliverables.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,7 +632,9 @@
         <v>5</v>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0.9980237154150198</v>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1141,7 +1143,9 @@
       <c r="F22" t="n">
         <v>6</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>22.36</v>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1533,7 +1537,9 @@
       <c r="J34" t="n">
         <v>2.78</v>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2398,7 +2404,9 @@
       <c r="J61" t="n">
         <v>7.18</v>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2802,10 +2810,10 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F74" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
@@ -2833,10 +2841,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F75" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
@@ -2856,22 +2864,20 @@
         </is>
       </c>
       <c r="C76" t="n">
+        <v>4</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>P4 - Stakeholder Responsiveness</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="n">
         <v>3</v>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>P3 - Employee Well-being</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>0</v>
-      </c>
-      <c r="F76" t="n">
-        <v>5</v>
-      </c>
-      <c r="G76" t="n">
-        <v>15.6</v>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
@@ -2889,21 +2895,23 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="n">
+        <v>0.0576299131121756</v>
+      </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr"/>
@@ -2920,23 +2928,21 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="n">
-        <v>0.0576299131121756</v>
-      </c>
+      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
@@ -2953,30 +2959,24 @@
         </is>
       </c>
       <c r="C79" t="n">
+        <v>8</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>P8 - Inclusive Growth</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>8</v>
+      </c>
+      <c r="F79" t="n">
         <v>6</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>P6 - Environment Protection</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" t="n">
-        <v>11</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
-      <c r="I79" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="J79" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="K79" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2990,18 +2990,18 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -3310,20 +3310,22 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F90" t="n">
-        <v>20</v>
-      </c>
-      <c r="G90" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>33.3</v>
+      </c>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr"/>
@@ -3341,18 +3343,18 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
@@ -3368,22 +3370,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E92" t="n">
         <v>0</v>
       </c>
       <c r="F92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
@@ -3399,22 +3401,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
@@ -3430,7 +3432,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -3442,10 +3444,10 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F94" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
@@ -3461,22 +3463,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C95" t="n">
+        <v>4</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>P4 - Stakeholder Responsiveness</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="n">
         <v>3</v>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>P3 - Employee Well-being</t>
-        </is>
-      </c>
-      <c r="E95" t="n">
-        <v>15</v>
-      </c>
-      <c r="F95" t="n">
-        <v>6</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
@@ -3492,25 +3494,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F96" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>0.8787860648868669</v>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
@@ -3523,28 +3527,32 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F97" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="J97" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0.02</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3554,34 +3562,28 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
-      <c r="I98" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="J98" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="K98" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3595,18 +3597,18 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
@@ -3626,18 +3628,18 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F100" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
@@ -3657,18 +3659,18 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
@@ -3679,29 +3681,31 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F102" t="n">
-        <v>2</v>
-      </c>
-      <c r="G102" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G102" t="n">
+        <v>32.5</v>
+      </c>
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
@@ -3710,27 +3714,27 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F103" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
@@ -3741,32 +3745,32 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F104" t="n">
         <v>6</v>
       </c>
-      <c r="G104" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>0.8772790599067175</v>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
@@ -3774,58 +3778,64 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
+      <c r="I105" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J105" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0.01</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F106" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
@@ -3836,39 +3846,33 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F107" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
-      <c r="I107" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="J107" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="K107" t="n">
-        <v>1.48</v>
-      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3882,18 +3886,18 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
@@ -3913,18 +3917,18 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -3944,20 +3948,22 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F110" t="n">
-        <v>13</v>
-      </c>
-      <c r="G110" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G110" t="n">
+        <v>3.66</v>
+      </c>
       <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
@@ -3971,22 +3977,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
@@ -4002,25 +4008,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F112" t="n">
         <v>5</v>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>0.06839945684696408</v>
+      </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
@@ -4033,30 +4041,34 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F113" t="n">
-        <v>6</v>
-      </c>
-      <c r="G113" t="n">
-        <v>3.26</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
+      <c r="I113" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J113" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="K113" t="n">
+        <v>1.48</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4066,22 +4078,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
@@ -4097,22 +4109,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
@@ -4128,34 +4140,28 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E116" t="n">
+        <v>10</v>
+      </c>
+      <c r="F116" t="n">
         <v>13</v>
-      </c>
-      <c r="F116" t="n">
-        <v>21</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
-      <c r="I116" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="J116" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="K116" t="n">
-        <v>0</v>
-      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4169,18 +4175,18 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
@@ -4200,18 +4206,18 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F118" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
@@ -4231,20 +4237,22 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F119" t="n">
-        <v>12</v>
-      </c>
-      <c r="G119" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G119" t="n">
+        <v>3.26</v>
+      </c>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
@@ -4258,22 +4266,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -4289,25 +4297,27 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F121" t="n">
         <v>5</v>
       </c>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
+      <c r="H121" t="n">
+        <v>0.06839946520106081</v>
+      </c>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr"/>
@@ -4320,30 +4330,34 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E122" t="n">
         <v>13</v>
       </c>
       <c r="F122" t="n">
-        <v>8</v>
-      </c>
-      <c r="G122" t="n">
-        <v>4.15</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
+      <c r="I122" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="K122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4353,22 +4367,22 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F123" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
@@ -4384,27 +4398,25 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" t="n">
-        <v>0.09473993638118393</v>
-      </c>
+      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr"/>
@@ -4417,31 +4429,27 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F125" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
-      <c r="I125" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="J125" t="n">
-        <v>0.08</v>
-      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
     </row>
     <row r="126">
@@ -4456,18 +4464,18 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -4487,15 +4495,15 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F127" t="n">
         <v>5</v>
@@ -4518,24 +4526,218 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F128" t="n">
-        <v>12</v>
-      </c>
-      <c r="G128" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="G128" t="n">
+        <v>4.15</v>
+      </c>
       <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>4</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>P4 - Stakeholder Responsiveness</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>2</v>
+      </c>
+      <c r="F129" t="n">
+        <v>3</v>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>5</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>P5 - Human Rights</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>11</v>
+      </c>
+      <c r="F130" t="n">
+        <v>5</v>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>0.09473993638118393</v>
+      </c>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>6</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>P6 - Environment Protection</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>13</v>
+      </c>
+      <c r="F131" t="n">
+        <v>8</v>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J131" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>7</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>P7 - Public Policy Advocacy</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>1</v>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>8</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>P8 - Inclusive Growth</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>5</v>
+      </c>
+      <c r="F133" t="n">
+        <v>5</v>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>9</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>P9 - Customer Responsibility</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>7</v>
+      </c>
+      <c r="F134" t="n">
+        <v>12</v>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4615,9 +4817,7 @@
       <c r="C2" t="n">
         <v>0.84</v>
       </c>
-      <c r="D2" t="n">
-        <v>0.66</v>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>1.44</v>
       </c>
@@ -4630,9 +4830,7 @@
       <c r="H2" t="n">
         <v>1.44</v>
       </c>
-      <c r="I2" t="n">
-        <v>0.611</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>5</v>
       </c>
@@ -4677,20 +4875,30 @@
           <t>Employee Turnover (%)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="n">
+        <v>22.36</v>
+      </c>
       <c r="C4" t="n">
         <v>10</v>
       </c>
       <c r="D4" t="n">
         <v>15.6</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>32.5</v>
+      </c>
       <c r="F4" t="n">
         <v>4.15</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="H4" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>16.922</v>
+      </c>
       <c r="J4" t="n">
         <v>5</v>
       </c>
@@ -4710,7 +4918,9 @@
       <c r="D5" t="n">
         <v>0.0576299131121756</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>0.8772790599067175</v>
+      </c>
       <c r="F5" t="n">
         <v>0.09473993638118393</v>
       </c>
@@ -4718,9 +4928,11 @@
         <v>-0.01451515355150864</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2092198223827346</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+        <v>0.8772790599067175</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2449</v>
+      </c>
       <c r="J5" t="n">
         <v>5</v>
       </c>
@@ -4835,9 +5047,7 @@
       <c r="C4" t="n">
         <v>0.76</v>
       </c>
-      <c r="D4" t="n">
-        <v>0.66</v>
-      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5033,7 +5243,9 @@
       <c r="C2" t="n">
         <v>25.5</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>22.36</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5076,8 +5288,12 @@
       <c r="B5" t="n">
         <v>39.6</v>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>32.5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5137,7 +5353,9 @@
           <t>AXIS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>0.9980237154150198</v>
+      </c>
       <c r="C2" t="n">
         <v>-0.008810961159019845</v>
       </c>
@@ -5187,9 +5405,11 @@
         <v>0.9985032740879326</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2046589018302828</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>0.8787860648868669</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8772790599067175</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5197,8 +5417,12 @@
           <t>PNB</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>0.06839945684696408</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.06839946520106081</v>
+      </c>
       <c r="D6" t="n">
         <v>0.09473993638118393</v>
       </c>
@@ -5259,7 +5483,9 @@
           <t>HDFC</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
       <c r="C3" t="n">
         <v>0.96</v>
       </c>
@@ -5273,7 +5499,9 @@
           <t>ICICI</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
       <c r="C4" t="n">
         <v>0.01</v>
       </c>
@@ -5322,7 +5550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7718,13 +7946,13 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F82" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G82" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="83">
@@ -7747,13 +7975,13 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F83" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G83" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
     </row>
     <row r="84">
@@ -7768,18 +7996,18 @@
         </is>
       </c>
       <c r="C84" t="n">
+        <v>4</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>P4 - Stakeholder Responsiveness</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="n">
         <v>3</v>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>P3 - Employee Well-being</t>
-        </is>
-      </c>
-      <c r="E84" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" t="n">
-        <v>5</v>
       </c>
       <c r="G84" t="n">
         <v>5</v>
@@ -7797,21 +8025,21 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F85" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G85" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="86">
@@ -7826,18 +8054,18 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F86" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G86" t="n">
         <v>5</v>
@@ -7855,21 +8083,21 @@
         </is>
       </c>
       <c r="C87" t="n">
+        <v>8</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>P8 - Inclusive Growth</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>8</v>
+      </c>
+      <c r="F87" t="n">
         <v>6</v>
       </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>P6 - Environment Protection</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" t="n">
-        <v>11</v>
-      </c>
       <c r="G87" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="88">
@@ -7884,21 +8112,21 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G88" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="89">
@@ -7923,13 +8151,13 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="F89" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G89" t="n">
-        <v>78</v>
+        <v>142</v>
       </c>
     </row>
     <row r="90">
@@ -8236,21 +8464,21 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -8265,21 +8493,21 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -8293,24 +8521,22 @@
           <t>2024-2025</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
+      <c r="C102" t="n">
+        <v>7</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>ALL PRINCIPLES</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F102" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -8321,7 +8547,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -8333,13 +8559,13 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F103" t="n">
         <v>2</v>
       </c>
       <c r="G103" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="104">
@@ -8350,25 +8576,25 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F104" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G104" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="105">
@@ -8379,22 +8605,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F105" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G105" t="n">
         <v>5</v>
@@ -8408,25 +8634,25 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F106" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G106" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="107">
@@ -8437,25 +8663,25 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G107" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108">
@@ -8466,25 +8692,25 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F108" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G108" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="109">
@@ -8495,25 +8721,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2025-2026</t>
-        </is>
-      </c>
-      <c r="C109" t="n">
-        <v>6</v>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>ALL PRINCIPLES</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F109" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="G109" t="n">
-        <v>7</v>
+        <v>90</v>
       </c>
     </row>
     <row r="110">
@@ -8528,21 +8756,21 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G110" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -8557,21 +8785,21 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F111" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112">
@@ -8586,21 +8814,21 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G112" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113">
@@ -8614,198 +8842,198 @@
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
+      <c r="C113" t="n">
+        <v>3</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ALL PRINCIPLES</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="F113" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="G113" t="n">
-        <v>103</v>
+        <v>21</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G114" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G115" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F116" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G116" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G117" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E118" t="n">
+        <v>7</v>
+      </c>
+      <c r="F118" t="n">
+        <v>4</v>
+      </c>
+      <c r="G118" t="n">
         <v>11</v>
-      </c>
-      <c r="F118" t="n">
-        <v>5</v>
-      </c>
-      <c r="G118" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>KOTAK</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2023-2024</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>6</v>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>ALL PRINCIPLES</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="F119" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="G119" t="n">
-        <v>20</v>
+        <v>86</v>
       </c>
     </row>
     <row r="120">
@@ -8820,21 +9048,21 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G120" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="121">
@@ -8849,21 +9077,21 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F121" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G121" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122">
@@ -8878,21 +9106,21 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F122" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G122" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="123">
@@ -8906,24 +9134,22 @@
           <t>2023-2024</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
+      <c r="C123" t="n">
+        <v>4</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>ALL PRINCIPLES</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="F123" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="G123" t="n">
-        <v>113</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
@@ -8934,25 +9160,25 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F124" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G124" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="125">
@@ -8963,25 +9189,25 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F125" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G125" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="126">
@@ -8992,25 +9218,25 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F126" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G126" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -9021,25 +9247,25 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E127" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F127" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G127" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="128">
@@ -9050,25 +9276,25 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F128" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G128" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="129">
@@ -9079,25 +9305,27 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2024-2025</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>6</v>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>ALL PRINCIPLES</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="F129" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="G129" t="n">
-        <v>34</v>
+        <v>113</v>
       </c>
     </row>
     <row r="130">
@@ -9112,21 +9340,21 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G130" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="131">
@@ -9141,21 +9369,21 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F131" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G131" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132">
@@ -9170,21 +9398,21 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E132" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F132" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G132" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="133">
@@ -9198,24 +9426,22 @@
           <t>2024-2025</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
+      <c r="C133" t="n">
+        <v>4</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>ALL PRINCIPLES</t>
+          <t>P4 - Stakeholder Responsiveness</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="F133" t="n">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="G133" t="n">
-        <v>126</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134">
@@ -9226,25 +9452,25 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>P1 - Ethics &amp; Transparency</t>
+          <t>P5 - Human Rights</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F134" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G134" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="135">
@@ -9255,25 +9481,25 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>P2 - Product Responsibility</t>
+          <t>P6 - Environment Protection</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F135" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="G135" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
     </row>
     <row r="136">
@@ -9284,25 +9510,25 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>P3 - Employee Well-being</t>
+          <t>P7 - Public Policy Advocacy</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G136" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -9313,25 +9539,25 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>P4 - Stakeholder Responsiveness</t>
+          <t>P8 - Inclusive Growth</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F137" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G137" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="138">
@@ -9342,25 +9568,25 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>P5 - Human Rights</t>
+          <t>P9 - Customer Responsibility</t>
         </is>
       </c>
       <c r="E138" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F138" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G138" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="139">
@@ -9371,25 +9597,27 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2025-2026</t>
-        </is>
-      </c>
-      <c r="C139" t="n">
-        <v>6</v>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>P6 - Environment Protection</t>
+          <t>ALL PRINCIPLES</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="F139" t="n">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="G139" t="n">
-        <v>21</v>
+        <v>126</v>
       </c>
     </row>
     <row r="140">
@@ -9404,21 +9632,21 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>P7 - Public Policy Advocacy</t>
+          <t>P1 - Ethics &amp; Transparency</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G140" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="141">
@@ -9433,21 +9661,21 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>P8 - Inclusive Growth</t>
+          <t>P2 - Product Responsibility</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F141" t="n">
         <v>5</v>
       </c>
       <c r="G141" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="142">
@@ -9462,21 +9690,21 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>P9 - Customer Responsibility</t>
+          <t>P3 - Employee Well-being</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F142" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G142" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="143">
@@ -9490,23 +9718,197 @@
           <t>2025-2026</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C143" t="n">
+        <v>4</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>P4 - Stakeholder Responsiveness</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>2</v>
+      </c>
+      <c r="F143" t="n">
+        <v>3</v>
+      </c>
+      <c r="G143" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>5</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>P5 - Human Rights</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>11</v>
+      </c>
+      <c r="F144" t="n">
+        <v>5</v>
+      </c>
+      <c r="G144" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>6</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>P6 - Environment Protection</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>13</v>
+      </c>
+      <c r="F145" t="n">
+        <v>8</v>
+      </c>
+      <c r="G145" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>7</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>P7 - Public Policy Advocacy</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>8</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>P8 - Inclusive Growth</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>5</v>
+      </c>
+      <c r="F147" t="n">
+        <v>5</v>
+      </c>
+      <c r="G147" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>9</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>P9 - Customer Responsibility</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>7</v>
+      </c>
+      <c r="F148" t="n">
+        <v>12</v>
+      </c>
+      <c r="G148" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr">
+      <c r="D149" t="inlineStr">
         <is>
           <t>ALL PRINCIPLES</t>
         </is>
       </c>
-      <c r="E143" t="n">
+      <c r="E149" t="n">
         <v>64</v>
       </c>
-      <c r="F143" t="n">
+      <c r="F149" t="n">
         <v>49</v>
       </c>
-      <c r="G143" t="n">
+      <c r="G149" t="n">
         <v>113</v>
       </c>
     </row>

</xml_diff>